<commit_message>
Tambah 3 plan khusus dalam kota Jogja (bunga, jurnal, galeri & foto)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jq83CRHReCm7A72dG1FuKN
</commit_message>
<xml_diff>
--- a/rencana-jogja/Rencana_Jalan-Jalan_Jogja_3Okt2026.xlsx
+++ b/rencana-jogja/Rencana_Jalan-Jalan_Jogja_3Okt2026.xlsx
@@ -14,6 +14,9 @@
     <sheet name="Membuat Keramik" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Meracik Parfum" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Candi &amp; Senja" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Merangkai Bunga" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Jurnal Kenangan" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Galeri &amp; Foto" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -576,6 +579,7 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,6 +647,11 @@
           <t>Wajib booking?</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Wilayah</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -683,6 +692,11 @@
           <t>Ya — workshop perak H-3</t>
         </is>
       </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Kota + Kotagede</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -723,6 +737,11 @@
           <t>Tidak (opsional tur museum)</t>
         </is>
       </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Utara (Sleman/Kaliurang)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -763,6 +782,11 @@
           <t>Ya — kelas batik</t>
         </is>
       </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Kota (Keraton–Prawirotaman)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -803,6 +827,11 @@
           <t>Ya — workshop keramik</t>
         </is>
       </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Selatan (Bantul)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -843,6 +872,11 @@
           <t>Ya — workshop parfum</t>
         </is>
       </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Kota + Adisucipto</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -883,64 +917,212 @@
           <t>Tidak (siapkan instax)</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Timur (Prambanan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Merangkai Bunga</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Buket yang kamu rangkai untuknya + kartu tulisan tangan.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="6">
+        <f>SUM(C11:G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>'Merangkai Bunga'!I17</f>
+        <v/>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Ya — kelas bunga privat</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>DALAM KOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Jurnal Kenangan</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Jurnal (kulit/handmade) yang halaman pertamanya sudah kamu isi dengan kenangan persahabatan kalian.</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="6">
+        <f>SUM(C12:G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="7">
+        <f>'Jurnal Kenangan'!I16</f>
+        <v/>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Tidak (siapkan jurnal dari rumah)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>DALAM KOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Galeri &amp; Foto</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Cetak foto terbaik kalian dari self-photo studio, masukkan ke bingkai kecil, dan tulis pesan di balik foto.</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="6">
+        <f>SUM(C13:G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="7">
+        <f>'Galeri &amp; Foto'!I17</f>
+        <v/>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Ya — slot studio foto H-1</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>DALAM KOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Catatan</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>• Skor 1–5 per kriteria adalah penilaian subjektif planner (bukan data Google Maps). Skor total dihitung otomatis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>• Rekomendasi utama: Plan 1 (hadiah paling tahan lama &amp; semua preferensi terpenuhi). Cadangan: Plan 5 (paling praktis) atau Plan 2 (paling tenang).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>• Status Info di tiap sheet: 'Terverifikasi' = dicek dari sumber web resmi/terbaru (Sep 2026); 'Perlu cek' = dari pengetahuan umum — buka link Google Maps &amp; cek jam buka H-1.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>• Biaya adalah ESTIMASI per orang (termasuk porsi transport). Edit kolom 'Est. Biaya' di tiap sheet — total &amp; ringkasan ikut berubah.</t>
+          <t>• Skor 1–5 per kriteria adalah penilaian subjektif planner (bukan data Google Maps). Skor total dihitung otomatis.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>• Cuaca: awal Oktober = peralihan ke musim hujan. Bawa payung lipat; untuk plan outdoor (4 &amp; 6) siapkan Plan B indoor.</t>
+          <t>• Rekomendasi utama: Plan 1 (hadiah paling tahan lama &amp; semua preferensi terpenuhi). Cadangan: Plan 5 (paling praktis) atau Plan 2 (paling tenang).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
+          <t>• Plan 7–9 = DALAM KOTA saja (perpindahan antar titik ±10–20 menit, tanpa naik ke Kaliurang/Bantul/Prambanan). Pilihan terbaik dalam kota: Plan 7 (Merangkai Bunga) atau Plan 9 (Galeri &amp; Foto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>• Status Info di tiap sheet: 'Terverifikasi' = dicek dari sumber web resmi/terbaru (Sep 2026); 'Perlu cek' = dari pengetahuan umum — buka link Google Maps &amp; cek jam buka H-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>• Biaya adalah ESTIMASI per orang (termasuk porsi transport). Edit kolom 'Est. Biaya' di tiap sheet — total &amp; ringkasan ikut berubah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>• Cuaca: awal Oktober = peralihan ke musim hujan. Bawa payung lipat; untuk plan outdoor (4 &amp; 6) siapkan Plan B indoor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
           <t>• Matahari terbenam di Jogja ±17.30 WIB — jadwal sudah disusun agar selesai sebelum 18.00.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A18:J18"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A13:J13"/>
+  <mergeCells count="7">
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A18:K18"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>
@@ -949,6 +1131,737 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId9"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan 9 (Dalam Kota) — Galeri, Studio Foto &amp; Cheesecake</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Konsep</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n"/>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Rute timur-tengah kota (Kotabaru – Adisucipto – Demangan – Terban), semua ≤15 menit. Museum seni, sesi self-photo studio, galeri fotografi sambil ngopi, tutup dengan basque cheesecake.</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="11" t="n"/>
+      <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Hadiah</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Cetak foto terbaik kalian dari self-photo studio, masukkan ke bingkai kecil, dan tulis pesan di balik foto. Cepat jadi hari itu juga, dan berbentuk benda yang dipajang — bukan disimpan di laci.</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="14" t="n"/>
+      <c r="L3" s="14" t="n"/>
+      <c r="M3" s="14" t="n"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Kenapa plan ini</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Semua preferensinya terpenuhi (latte, roti, cheesecake, tenang). Titik lemah: nama studio foto tidak kutentukan — pilih yang ratingnya bagus di Maps.</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mulai</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Durasi (menit)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Aktivitas</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Tempat</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Alamat / Area</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Est. Biaya / Orang (Rp)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Transport dari titik sebelumnya</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Kenapa cocok untuk dia</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Tips / Catatan</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Status Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="D7" s="16">
+        <f>ROUND((C7-B7)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Sarapan: roti savory + latte</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Cosan Coffee Kotabaru</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Pattimura, Kotabaru</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Titik awal</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Buka sejak pagi, sepi di jam 9.</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Buka 06.00–24.00.</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>Terverifikasi (TikTok info cabang)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D8" s="16">
+        <f>ROUND((C8-B8)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Museum Affandi</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±4 km</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="16">
+        <f>ROUND((C9-B9)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Museum Affandi</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Museum Affandi</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Laksda Adisucipto 167</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Galeri tenang di tepi Kali Gajah Wong.</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Konfirmasi jam buka Sabtu di Maps.</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>0.5520833333333334</v>
+      </c>
+      <c r="D10" s="16">
+        <f>ROUND((C10-B10)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Makan siang</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>Pilihan bebas area Demangan/Gejayan</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>Demangan</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±2 km</t>
+        </is>
+      </c>
+      <c r="K10" s="16" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>0.6145833333333334</v>
+      </c>
+      <c r="D11" s="16">
+        <f>ROUND((C11-B11)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>SESI SELF-PHOTO STUDIO + cetak &amp; bingkai</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Self-photo studio (pilih di Maps)</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Area Demangan/Gejayan</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±10 mnt</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Seru, privat (tanpa fotografer), hasil langsung dicetak.</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Booking slot online H-1; bawa/ beli bingkai kecil.</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>0.6145833333333334</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D12" s="16">
+        <f>ROUND((C12-B12)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Terban</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±3 km</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr"/>
+      <c r="L12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="D13" s="16">
+        <f>ROUND((C13-B13)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Galeri fotografi + latte; tulis pesan di balik foto</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Awor Gallery &amp; Coffee</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Jl. C. Simanjuntak, Ruko Yap Square 11B, Terban</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Kafe sekaligus galeri foto — nyambung dengan tema hadiah.</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Buka ±08.00/09.00–23.00/24.00.</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Terverifikasi (Tripadvisor, jogjasuper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="D14" s="16">
+        <f>ROUND((C14-B14)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Demangan</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr"/>
+      <c r="H14" s="16" t="n"/>
+      <c r="I14" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±2 km</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr"/>
+      <c r="L14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>0.7395833333333334</v>
+      </c>
+      <c r="D15" s="19">
+        <f>ROUND((C15-B15)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Basque burnt cheesecake. Serahkan foto berbingkai.</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Cosan Coffee Demangan</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>Demangan</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>Cheesecake-nya jadi incaran.</t>
+        </is>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>Pilih meja pojok.</t>
+        </is>
+      </c>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>Sebagian terverifikasi (IG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>0.7395833333333334</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D16" s="16">
+        <f>ROUND((C16-B16)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Penutup</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr"/>
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J16" s="16" t="inlineStr"/>
+      <c r="K16" s="16" t="inlineStr"/>
+      <c r="L16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="n"/>
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24">
+        <f>SUM(D7:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
+      <c r="H17" s="24" t="n"/>
+      <c r="I17" s="25">
+        <f>SUM(I7:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>per orang (estimasi)</t>
+        </is>
+      </c>
+      <c r="K17" s="24" t="n"/>
+      <c r="L17" s="24" t="n"/>
+      <c r="M17" s="24" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Baris merah muda = momen workshop/hadiah. Angka biru = estimasi yang boleh kamu ubah. Link 'Buka Maps' membuka pencarian Google Maps untuk tempat tsb.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C4:M4"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="C2:M2"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4787,4 +5700,1422 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan 7 (Dalam Kota) — Merangkai Bunga di Kotabaru</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Konsep</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n"/>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Semua titik di dalam kota, perpindahan maks ±15 menit. Pagi di Kotabaru yang teduh, kelas merangkai bunga privat (maks 2 orang), museum ber-AC di siang terik, lalu cheesecake di Mangkubumi.</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="11" t="n"/>
+      <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Hadiah</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Buket yang kamu rangkai untuknya + kartu tulisan tangan. Karena bunga segar layu, sisihkan 1 tangkai untuk dikeringkan (pressed flower) — dia bisa menyimpannya di buku/bingkai kecil.</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="14" t="n"/>
+      <c r="L3" s="14" t="n"/>
+      <c r="M3" s="14" t="n"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Kenapa plan ini</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Kelas privat = suasana tenang &amp; intim tanpa orang asing. Harga kelas dari situs resmi. Titik lemah: alamat studio baru diberikan saat reservasi.</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mulai</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Durasi (menit)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Aktivitas</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Tempat</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Alamat / Area</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Est. Biaya / Orang (Rp)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Transport dari titik sebelumnya</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Kenapa cocok untuk dia</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Tips / Catatan</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Status Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="D7" s="16">
+        <f>ROUND((C7-B7)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Sarapan: roti/sandwich savory + caffe latte</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Cosan Coffee Kotabaru</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Pattimura, Kotabaru</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Titik awal</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Buka dari pagi; Kotabaru termasuk kawasan paling teduh &amp; tenang di pusat kota.</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Buka 06.00–24.00.</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>Terverifikasi (TikTok info cabang)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="D8" s="16">
+        <f>ROUND((C8-B8)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Jalan kaki heritage Kotabaru (rumah-rumah indis, Gereja St. Antonius)</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>Kawasan Cagar Budaya Kotabaru</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Kotabaru</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>Jalan kaki</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>Jalanan rindang, sepi di Sabtu pagi — enak untuk ngobrol.</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="D9" s="16">
+        <f>ROUND((C9-B9)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke studio bunga</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr"/>
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Ojol (alamat dari admin)</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>0.5520833333333334</v>
+      </c>
+      <c r="D10" s="19">
+        <f>ROUND((C10-B10)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>KELAS MERANGKAI BUNGA — Private Hobby Class (1–2 orang, 90–120 mnt)</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Bebungaan Atelier</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Konfirmasi saat reservasi</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>385000</v>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>Konsep 'atmospheric storytelling' lewat bunga; semua bahan disediakan.</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>Harga mulai Rp385rb/orang (private). Booking via bebungaan.com. Alternatif: Hanabira / Kirei Florist (±Rp150–250rb).</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Terverifikasi (bebungaan.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0.5520833333333334</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="D11" s="16">
+        <f>ROUND((C11-B11)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Makan siang</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Pilihan bebas area Kotabaru/Jl. Suroto</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Kotabaru</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±10 mnt</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr"/>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Titipkan buket di mobil/tempat teduh.</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0.6041666666666666</v>
+      </c>
+      <c r="D12" s="16">
+        <f>ROUND((C12-B12)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Sonobudoyo</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±3 km</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr"/>
+      <c r="L12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>0.6041666666666666</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="D13" s="16">
+        <f>ROUND((C13-B13)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Museum Sonobudoyo Unit I (keris, wayang, topeng, naskah kuno)</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Museum Sonobudoyo</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Pangurakan / Trikora, utara Alun-alun</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>Ber-AC, tertata rapi, tidak berisik — pelarian dari panas siang.</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Buka Sel–Min 08.00–21.00, tiket dewasa Rp10rb.</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Terverifikasi (sonobudoyo.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>0.6770833333333334</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>0.6909722222222222</v>
+      </c>
+      <c r="D14" s="16">
+        <f>ROUND((C14-B14)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Jl. Mangkubumi</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr"/>
+      <c r="H14" s="16" t="n"/>
+      <c r="I14" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±3 km</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr"/>
+      <c r="L14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>0.6909722222222222</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="D15" s="19">
+        <f>ROUND((C15-B15)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Cheesecake + latte. Serahkan buket &amp; kartu.</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Roaster and Bear</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>Jl. P. Mangkubumi No.52</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="n">
+        <v>90000</v>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>Cheesecake termasuk menu paling direkomendasikan.</t>
+        </is>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>Sore Sabtu ramai — minta meja dalam/pojok.</t>
+        </is>
+      </c>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>Terverifikasi (Tripadvisor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D16" s="16">
+        <f>ROUND((C16-B16)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Penutup (dekat Tugu)</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr"/>
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="16" t="inlineStr"/>
+      <c r="K16" s="16" t="inlineStr"/>
+      <c r="L16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="n"/>
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24">
+        <f>SUM(D7:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
+      <c r="H17" s="24" t="n"/>
+      <c r="I17" s="25">
+        <f>SUM(I7:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
+        <is>
+          <t>per orang (estimasi)</t>
+        </is>
+      </c>
+      <c r="K17" s="24" t="n"/>
+      <c r="L17" s="24" t="n"/>
+      <c r="M17" s="24" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Baris merah muda = momen workshop/hadiah. Angka biru = estimasi yang boleh kamu ubah. Link 'Buka Maps' membuka pencarian Google Maps untuk tempat tsb.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C4:M4"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="C2:M2"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan 8 (Dalam Kota) — Jurnal Kenangan di Njeron Beteng &amp; Prawirotaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Konsep</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n"/>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Kawasan selatan kota yang bisa dijelajah dengan jalan kaki/ojol singkat: bakery Tirtodipuran, Keraton, galeri &amp; toko zine, lalu sesi journaling santai di ViaVia sambil latte.</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="11" t="n"/>
+      <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Hadiah</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Jurnal (kulit/handmade) yang halaman pertamanya sudah kamu isi dengan kenangan persahabatan kalian. Sepanjang hari kumpulkan tiket, stiker, struk — lalu tempel bersama di sesi terakhir. Siapkan jurnal &amp; perlengkapan (lem, gunting kecil, washi tape) SEBELUM hari H.</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="14" t="n"/>
+      <c r="L3" s="14" t="n"/>
+      <c r="M3" s="14" t="n"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Kenapa plan ini</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Paling murah &amp; paling personal; tidak bergantung pada slot workshop. Titik lemah: cheesecake tidak terjamin di rute ini.</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mulai</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Durasi (menit)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Aktivitas</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Tempat</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Alamat / Area</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Est. Biaya / Orang (Rp)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Transport dari titik sebelumnya</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Kenapa cocok untuk dia</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Tips / Catatan</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Status Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="D7" s="16">
+        <f>ROUND((C7-B7)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Sarapan: croissant, quiche/roti savory + latte</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Mediterranea Store &amp; Bakery</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Tirtodipuran No.24</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Titik awal</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>Roti savory kuat; tenang di pagi hari.</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Buka 08.00.</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>Terverifikasi (IG resmi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D8" s="16">
+        <f>ROUND((C8-B8)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Keraton</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±3 km</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+      <c r="D9" s="16">
+        <f>ROUND((C9-B9)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Keraton Yogyakarta (Kedhaton)</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Keraton Ngayogyakarta Hadiningrat</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Rotowijayan</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>Ikon Jogja; simpan tiketnya untuk jurnal.</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Umumnya tutup ±14.00 — makanya dijadwalkan pagi. Cek jam &amp; tiket terbaru.</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>0.5069444444444444</v>
+      </c>
+      <c r="D10" s="16">
+        <f>ROUND((C10-B10)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Perjalanan ke Tirtodipuran</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±2 km</t>
+        </is>
+      </c>
+      <c r="K10" s="16" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0.5069444444444444</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="D11" s="16">
+        <f>ROUND((C11-B11)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Makan siang masakan Jawa rumahan</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Warung Bu Ageng</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Tirtodipuran</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Tenang, suasana rumah Jawa.</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D12" s="16">
+        <f>ROUND((C12-B12)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Galeri &amp; toko buku/zine — cari stiker, kartu pos, zine untuk jurnal</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Kedai Kebun Forum &amp; galeri sepanjang Tirtodipuran</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Jl. Tirtodipuran</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Jalan kaki</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>Ruang seni kecil yang sepi; pas untuk 'berburu' isi jurnal.</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>Biaya = belanja kecil (kartu pos, zine).</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>0.6354166666666666</v>
+      </c>
+      <c r="D13" s="16">
+        <f>ROUND((C13-B13)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Pindah ke Prawirotaman</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr"/>
+      <c r="H13" s="16" t="n"/>
+      <c r="I13" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±1,5 km</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr"/>
+      <c r="L13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>0.6354166666666666</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="D14" s="19">
+        <f>ROUND((C14-B14)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>SESI JOURNALING: tempel koleksi hari ini, tulis bersama + latte &amp; kue. Serahkan jurnal.</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>ViaVia Jogja</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>Jl. Prawirotaman</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="n">
+        <v>90000</v>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>Kafe santai dengan artisan bakery; ViaVia juga kadang mengadakan kelas bookbinding &amp; journaling (#ViaViaSinau).</t>
+        </is>
+      </c>
+      <c r="L14" s="19" t="inlineStr">
+        <is>
+          <t>Cek IG/web ViaVia: kalau kebetulan ada kelas bookbinding di tanggal itu, ikuti.</t>
+        </is>
+      </c>
+      <c r="M14" s="19" t="inlineStr">
+        <is>
+          <t>Sebagian terverifikasi (viaviajogja.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D15" s="16">
+        <f>ROUND((C15-B15)*1440,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Jalan santai sore menuju Pojok Beteng Kulon (senja ±17.30)</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Pojok Beteng Kulon</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Patehan, Kraton</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Buka Maps</t>
+        </is>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Ojol ±2 km</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>Senja di benteng tua — penutup yang tenang.</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr"/>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>Perlu cek</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="n"/>
+      <c r="B16" s="24" t="n"/>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24">
+        <f>SUM(D7:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="n"/>
+      <c r="G16" s="24" t="n"/>
+      <c r="H16" s="24" t="n"/>
+      <c r="I16" s="25">
+        <f>SUM(I7:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="24" t="inlineStr">
+        <is>
+          <t>per orang (estimasi)</t>
+        </is>
+      </c>
+      <c r="K16" s="24" t="n"/>
+      <c r="L16" s="24" t="n"/>
+      <c r="M16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Baris merah muda = momen workshop/hadiah. Angka biru = estimasi yang boleh kamu ubah. Link 'Buka Maps' membuka pencarian Google Maps untuk tempat tsb.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C4:M4"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="C2:M2"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>